<commit_message>
update readme file. update point labels.
</commit_message>
<xml_diff>
--- a/summary output/point_labels_all(readme).xlsx
+++ b/summary output/point_labels_all(readme).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pjs23\Documents\R\slash-wall-vegetation\summary output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6362B52C-3FA5-4D30-92C8-F4C647716C48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A687C2A-FA6E-4FC9-9753-80ED705909DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10391" uniqueCount="708">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10392" uniqueCount="709">
   <si>
     <t>harvest</t>
   </si>
@@ -2159,6 +2159,9 @@
   </si>
   <si>
     <t>u</t>
+  </si>
+  <si>
+    <t>Scope - these data pertain to slash walls created between 2017 and 2022 and can match all attributes by point numbers, which are unique.</t>
   </si>
 </sst>
 </file>
@@ -40677,54 +40680,59 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3559735D-14BA-4E17-B1BD-46A6A98F1E0A}">
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="136.140625" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
-        <v>693</v>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
+        <v>708</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
         <v>700</v>
       </c>
     </row>

</xml_diff>

<commit_message>
lots of new code
</commit_message>
<xml_diff>
--- a/summary output/point_labels_all(readme).xlsx
+++ b/summary output/point_labels_all(readme).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pjs23\Documents\R\slash-wall-vegetation\summary output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A687C2A-FA6E-4FC9-9753-80ED705909DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22ECF16A-6DFB-4706-B39A-899E9CD26C7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>